<commit_message>
Actualizar archivos de VILGAR
</commit_message>
<xml_diff>
--- a/public/catalogo.xlsx
+++ b/public/catalogo.xlsx
@@ -4,17 +4,22 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de Precios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validación 40%" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validación 40%'!$A$1:$J$86</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -30,8 +35,12 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +50,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,6 +167,18 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -456,8 +487,8 @@
           <t>NOW DESENGRASANTE MULTIUSOS 1 L</t>
         </is>
       </c>
-      <c r="C2" s="26" t="n">
-        <v>75.23999999999999</v>
+      <c r="C2" s="31" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="3">
@@ -471,8 +502,8 @@
           <t>NOW DESENGRASANTE MULTIUSOS 5/1 L</t>
         </is>
       </c>
-      <c r="C3" s="26" t="n">
-        <v>195.36</v>
+      <c r="C3" s="31" t="n">
+        <v>205</v>
       </c>
     </row>
     <row r="4">
@@ -486,8 +517,8 @@
           <t>NOW DESENGRASANTE MULTIUSOS 20 L</t>
         </is>
       </c>
-      <c r="C4" s="26" t="n">
-        <v>580.8</v>
+      <c r="C4" s="31" t="n">
+        <v>581</v>
       </c>
     </row>
     <row r="5">
@@ -501,8 +532,8 @@
           <t>NOW DESENGRASANTE MULTIUSOS 208 L</t>
         </is>
       </c>
-      <c r="C5" s="26" t="n">
-        <v>5563.8</v>
+      <c r="C5" s="31" t="n">
+        <v>5811</v>
       </c>
     </row>
     <row r="6">
@@ -516,8 +547,8 @@
           <t>NOW DESENGRASANTE MULTIUSOS 1000 L</t>
         </is>
       </c>
-      <c r="C6" s="26" t="n">
-        <v>15557.52</v>
+      <c r="C6" s="31" t="n">
+        <v>16276</v>
       </c>
     </row>
     <row r="7">
@@ -531,8 +562,8 @@
           <t>NOW DESENGRASANTE COCINAS 1 L</t>
         </is>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>75.23999999999999</v>
+      <c r="C7" s="31" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="8">
@@ -546,8 +577,8 @@
           <t>NOW DESENGRASANTE DE COCINA 208 L</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
-        <v>5563.8</v>
+      <c r="C8" s="31" t="n">
+        <v>5811</v>
       </c>
     </row>
     <row r="9">
@@ -561,8 +592,8 @@
           <t>NOW DESENGRASANTE DE COCINA 1000 L</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n">
-        <v>15557.52</v>
+      <c r="C9" s="31" t="n">
+        <v>16276</v>
       </c>
     </row>
     <row r="10">
@@ -576,8 +607,8 @@
           <t>NOW VIDRIOS Y SUPERFICIES 1 L</t>
         </is>
       </c>
-      <c r="C10" s="26" t="n">
-        <v>75.23999999999999</v>
+      <c r="C10" s="31" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="11">
@@ -591,8 +622,8 @@
           <t>NOW VIDRIOS Y SUPERFICIES 5/1 L</t>
         </is>
       </c>
-      <c r="C11" s="26" t="n">
-        <v>195.36</v>
+      <c r="C11" s="31" t="n">
+        <v>205</v>
       </c>
     </row>
     <row r="12">
@@ -606,8 +637,8 @@
           <t>NOW VIDRIOS Y SUPERFICIES 208 L</t>
         </is>
       </c>
-      <c r="C12" s="26" t="n">
-        <v>3979.8</v>
+      <c r="C12" s="31" t="n">
+        <v>4148</v>
       </c>
     </row>
     <row r="13">
@@ -621,8 +652,8 @@
           <t>NOW VIDRIOS Y SUPERFICIES 1000 L</t>
         </is>
       </c>
-      <c r="C13" s="26" t="n">
-        <v>10845.12</v>
+      <c r="C13" s="31" t="n">
+        <v>11211</v>
       </c>
     </row>
     <row r="14">
@@ -636,8 +667,8 @@
           <t>NOW DETERGENTE 1 L</t>
         </is>
       </c>
-      <c r="C14" s="26" t="n">
-        <v>42.24</v>
+      <c r="C14" s="31" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="15">
@@ -651,8 +682,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 5 L MX</t>
         </is>
       </c>
-      <c r="C15" s="26" t="n">
-        <v>147.84</v>
+      <c r="C15" s="31" t="n">
+        <v>147</v>
       </c>
     </row>
     <row r="16">
@@ -666,8 +697,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 10 L</t>
         </is>
       </c>
-      <c r="C16" s="26" t="n">
-        <v>278.52</v>
+      <c r="C16" s="31" t="n">
+        <v>259</v>
       </c>
     </row>
     <row r="17">
@@ -681,8 +712,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 10 L DB</t>
         </is>
       </c>
-      <c r="C17" s="26" t="n">
-        <v>372.24</v>
+      <c r="C17" s="31" t="n">
+        <v>379</v>
       </c>
     </row>
     <row r="18">
@@ -696,8 +727,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 20 L</t>
         </is>
       </c>
-      <c r="C18" s="26" t="n">
-        <v>633.6</v>
+      <c r="C18" s="31" t="n">
+        <v>645</v>
       </c>
     </row>
     <row r="19">
@@ -711,8 +742,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 208 L</t>
         </is>
       </c>
-      <c r="C19" s="26" t="n">
-        <v>6961.68</v>
+      <c r="C19" s="31" t="n">
+        <v>7223</v>
       </c>
     </row>
     <row r="20">
@@ -726,8 +757,8 @@
           <t>NOW DETERGENTE LIQ ROPA COLOR 1000 L</t>
         </is>
       </c>
-      <c r="C20" s="26" t="n">
-        <v>18579</v>
+      <c r="C20" s="31" t="n">
+        <v>18641</v>
       </c>
     </row>
     <row r="21">
@@ -741,8 +772,8 @@
           <t>NOW BAÑOS Y AZULEJOS 1 L</t>
         </is>
       </c>
-      <c r="C21" s="26" t="n">
-        <v>75.23999999999999</v>
+      <c r="C21" s="31" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="22">
@@ -756,8 +787,8 @@
           <t>NOW BAÑOS Y AZULEJOS 5+1 L</t>
         </is>
       </c>
-      <c r="C22" s="26" t="n">
-        <v>195.36</v>
+      <c r="C22" s="31" t="n">
+        <v>205</v>
       </c>
     </row>
     <row r="23">
@@ -771,8 +802,8 @@
           <t>NOW BAÑOS Y AZULEJOS 20 L</t>
         </is>
       </c>
-      <c r="C23" s="26" t="n">
-        <v>580.8</v>
+      <c r="C23" s="31" t="n">
+        <v>581</v>
       </c>
     </row>
     <row r="24">
@@ -786,8 +817,8 @@
           <t>NOW BAÑOS Y AZULEJOS 208 L</t>
         </is>
       </c>
-      <c r="C24" s="26" t="n">
-        <v>5563.8</v>
+      <c r="C24" s="31" t="n">
+        <v>5811</v>
       </c>
     </row>
     <row r="25">
@@ -801,8 +832,8 @@
           <t>NOW BAÑOS Y AZULEJOS 1000 L</t>
         </is>
       </c>
-      <c r="C25" s="26" t="n">
-        <v>15557.52</v>
+      <c r="C25" s="31" t="n">
+        <v>16276</v>
       </c>
     </row>
     <row r="26">
@@ -816,8 +847,8 @@
           <t>NOW SHAMPOO AUTOMOTRIZ 10 L (PEAD)</t>
         </is>
       </c>
-      <c r="C26" s="26" t="n">
-        <v>212.52</v>
+      <c r="C26" s="31" t="n">
+        <v>221</v>
       </c>
     </row>
     <row r="27">
@@ -831,8 +862,8 @@
           <t>NOW SHAMPOO AUTOMOTRIZ 10 L (PET)</t>
         </is>
       </c>
-      <c r="C27" s="26" t="n">
-        <v>163.68</v>
+      <c r="C27" s="31" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="28">
@@ -846,8 +877,8 @@
           <t>NOW SHAMPOO AUTOMOTRIZ 208 L</t>
         </is>
       </c>
-      <c r="C28" s="26" t="n">
-        <v>4762.56</v>
+      <c r="C28" s="31" t="n">
+        <v>4964</v>
       </c>
     </row>
     <row r="29">
@@ -861,8 +892,8 @@
           <t>NOW SHAMPOO P/AUTO 1000 L</t>
         </is>
       </c>
-      <c r="C29" s="26" t="n">
-        <v>10879.44</v>
+      <c r="C29" s="31" t="n">
+        <v>11341</v>
       </c>
     </row>
     <row r="30">
@@ -876,8 +907,8 @@
           <t>NOW ABRILLANTADOR P/AUTO 1 L ATOM</t>
         </is>
       </c>
-      <c r="C30" s="26" t="n">
-        <v>62.04</v>
+      <c r="C30" s="31" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="31">
@@ -891,8 +922,8 @@
           <t>NOW ABRILLANTADOR P/AUTO 5/1 L</t>
         </is>
       </c>
-      <c r="C31" s="26" t="n">
-        <v>273.24</v>
+      <c r="C31" s="31" t="n">
+        <v>284</v>
       </c>
     </row>
     <row r="32">
@@ -906,8 +937,8 @@
           <t>NOW ABRILLANTADOR P/AUTO 20 L</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>777.48</v>
+      <c r="C32" s="31" t="n">
+        <v>812</v>
       </c>
     </row>
     <row r="33">
@@ -921,8 +952,8 @@
           <t>NOW ABRILLANTADOR P/AUTO 208 L</t>
         </is>
       </c>
-      <c r="C33" s="26" t="n">
-        <v>8125.92</v>
+      <c r="C33" s="31" t="n">
+        <v>8471</v>
       </c>
     </row>
     <row r="34">
@@ -936,8 +967,8 @@
           <t>NOW ABRILLANTADOR P/AUTO 1000 L</t>
         </is>
       </c>
-      <c r="C34" s="26" t="n">
-        <v>27556.32</v>
+      <c r="C34" s="31" t="n">
+        <v>28726</v>
       </c>
     </row>
     <row r="35">
@@ -951,8 +982,8 @@
           <t>NOW LAVATRASTES LIMON 2.90 L MX</t>
         </is>
       </c>
-      <c r="C35" s="26" t="n">
-        <v>137.28</v>
+      <c r="C35" s="31" t="n">
+        <v>144</v>
       </c>
     </row>
     <row r="36">
@@ -966,8 +997,8 @@
           <t>NOW LAVATRASTES LIMON 5 L</t>
         </is>
       </c>
-      <c r="C36" s="26" t="n">
-        <v>166.32</v>
+      <c r="C36" s="31" t="n">
+        <v>173</v>
       </c>
     </row>
     <row r="37">
@@ -981,8 +1012,8 @@
           <t>NOW LAVATRASTES 208 L</t>
         </is>
       </c>
-      <c r="C37" s="26" t="n">
-        <v>7975.44</v>
+      <c r="C37" s="31" t="n">
+        <v>8313</v>
       </c>
     </row>
     <row r="38">
@@ -996,8 +1027,8 @@
           <t>NOW LAVATRASTES 1000 L</t>
         </is>
       </c>
-      <c r="C38" s="26" t="n">
-        <v>25542</v>
+      <c r="C38" s="31" t="n">
+        <v>26623</v>
       </c>
     </row>
     <row r="39">
@@ -1011,8 +1042,8 @@
           <t>NOW LIMPIADOR PINO 1 L</t>
         </is>
       </c>
-      <c r="C39" s="26" t="n">
-        <v>34.32</v>
+      <c r="C39" s="31" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="40">
@@ -1026,8 +1057,8 @@
           <t>NOW LIMPIADOR PINO 5 L</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n">
-        <v>128.04</v>
+      <c r="C40" s="31" t="n">
+        <v>133</v>
       </c>
     </row>
     <row r="41">
@@ -1041,8 +1072,8 @@
           <t>NOW LIMPIADOR PINO 10 L</t>
         </is>
       </c>
-      <c r="C41" s="26" t="n">
-        <v>233.64</v>
+      <c r="C41" s="31" t="n">
+        <v>243</v>
       </c>
     </row>
     <row r="42">
@@ -1056,8 +1087,8 @@
           <t>NOW LIMPIADOR PINO 20 L</t>
         </is>
       </c>
-      <c r="C42" s="26" t="n">
-        <v>473.88</v>
+      <c r="C42" s="31" t="n">
+        <v>494</v>
       </c>
     </row>
     <row r="43">
@@ -1071,8 +1102,8 @@
           <t>NOW LIMPIADOR PINO 208 L</t>
         </is>
       </c>
-      <c r="C43" s="26" t="n">
-        <v>5772.36</v>
+      <c r="C43" s="31" t="n">
+        <v>6021</v>
       </c>
     </row>
     <row r="44">
@@ -1086,8 +1117,8 @@
           <t>NOW LIMPIADOR PINO 1000 L</t>
         </is>
       </c>
-      <c r="C44" s="26" t="n">
-        <v>16336.32</v>
+      <c r="C44" s="31" t="n">
+        <v>17035</v>
       </c>
     </row>
     <row r="45">
@@ -1101,8 +1132,8 @@
           <t>NOW LIMPIADOR MANZANA CANELA 1 L</t>
         </is>
       </c>
-      <c r="C45" s="26" t="n">
-        <v>31.68</v>
+      <c r="C45" s="31" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="46">
@@ -1116,8 +1147,8 @@
           <t>NOW LIMPIADOR MANZANA CANELA 5 L</t>
         </is>
       </c>
-      <c r="C46" s="26" t="n">
-        <v>99</v>
+      <c r="C46" s="31" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="47">
@@ -1131,8 +1162,8 @@
           <t>NOW LIMPIADOR MANZANA CANELA 10 L</t>
         </is>
       </c>
-      <c r="C47" s="26" t="n">
-        <v>161.04</v>
+      <c r="C47" s="31" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="48">
@@ -1146,8 +1177,8 @@
           <t>NOW QUITAMANCHAS GEL 10 L</t>
         </is>
       </c>
-      <c r="C48" s="26" t="n">
-        <v>293.04</v>
+      <c r="C48" s="31" t="n">
+        <v>306</v>
       </c>
     </row>
     <row r="49">
@@ -1161,8 +1192,8 @@
           <t>NOW QUITAMANCHAS 208 L</t>
         </is>
       </c>
-      <c r="C49" s="26" t="n">
-        <v>5491.2</v>
+      <c r="C49" s="31" t="n">
+        <v>5751</v>
       </c>
     </row>
     <row r="50">
@@ -1176,8 +1207,8 @@
           <t>NOW QUITAMANCHAS GEL 1000 L</t>
         </is>
       </c>
-      <c r="C50" s="26" t="n">
-        <v>15046.68</v>
+      <c r="C50" s="31" t="n">
+        <v>15696</v>
       </c>
     </row>
     <row r="51">
@@ -1191,8 +1222,8 @@
           <t>NOW DESENGRASANTE AUTOMOTRIZ 5 L</t>
         </is>
       </c>
-      <c r="C51" s="26" t="n">
-        <v>219.12</v>
+      <c r="C51" s="31" t="n">
+        <v>224</v>
       </c>
     </row>
     <row r="52">
@@ -1206,8 +1237,8 @@
           <t>NOW DESENGRASANTE AUTOMOTRIZ 20 L</t>
         </is>
       </c>
-      <c r="C52" s="26" t="n">
-        <v>851.4</v>
+      <c r="C52" s="31" t="n">
+        <v>889</v>
       </c>
     </row>
     <row r="53">
@@ -1221,8 +1252,8 @@
           <t>NOW DESENGRASANTE AUTOMOTRIZ 208 L</t>
         </is>
       </c>
-      <c r="C53" s="26" t="n">
-        <v>8511.360000000001</v>
+      <c r="C53" s="31" t="n">
+        <v>8881</v>
       </c>
     </row>
     <row r="54">
@@ -1236,8 +1267,8 @@
           <t>NOW DESENGRASANTE AUTOMOTRIZ 1000 L</t>
         </is>
       </c>
-      <c r="C54" s="26" t="n">
-        <v>32673.96</v>
+      <c r="C54" s="31" t="n">
+        <v>34230</v>
       </c>
     </row>
     <row r="55">
@@ -1251,8 +1282,8 @@
           <t>NOW LIMPIADOR BRISA MARINA 1 L</t>
         </is>
       </c>
-      <c r="C55" s="26" t="n">
-        <v>31.68</v>
+      <c r="C55" s="31" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="56">
@@ -1266,8 +1297,8 @@
           <t>NOW LIMPIADOR BRISA MARINA 5 L</t>
         </is>
       </c>
-      <c r="C56" s="26" t="n">
-        <v>99</v>
+      <c r="C56" s="31" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="57">
@@ -1281,8 +1312,8 @@
           <t>NOW LIMPIADOR BRISA DE MAR 10 L</t>
         </is>
       </c>
-      <c r="C57" s="26" t="n">
-        <v>161.04</v>
+      <c r="C57" s="31" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="58">
@@ -1296,8 +1327,8 @@
           <t>NOW LIMPIADOR LAVANDA 1 L</t>
         </is>
       </c>
-      <c r="C58" s="26" t="n">
-        <v>31.68</v>
+      <c r="C58" s="31" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="59">
@@ -1311,8 +1342,8 @@
           <t>NOW LIMPIADOR LAVANDA 5 L</t>
         </is>
       </c>
-      <c r="C59" s="26" t="n">
-        <v>93.72</v>
+      <c r="C59" s="31" t="n">
+        <v>98</v>
       </c>
     </row>
     <row r="60">
@@ -1326,8 +1357,8 @@
           <t>NOW LIMPIADOR LAVANDA 10 L</t>
         </is>
       </c>
-      <c r="C60" s="26" t="n">
-        <v>154.44</v>
+      <c r="C60" s="31" t="n">
+        <v>161</v>
       </c>
     </row>
     <row r="61">
@@ -1341,8 +1372,8 @@
           <t>NOW LIMPIADOR LAVANDA 20 L</t>
         </is>
       </c>
-      <c r="C61" s="26" t="n">
-        <v>370.92</v>
+      <c r="C61" s="31" t="n">
+        <v>386</v>
       </c>
     </row>
     <row r="62">
@@ -1356,8 +1387,8 @@
           <t>NOW LIMPIADOR LAVANDA 208 L</t>
         </is>
       </c>
-      <c r="C62" s="26" t="n">
-        <v>4675.44</v>
+      <c r="C62" s="31" t="n">
+        <v>4876</v>
       </c>
     </row>
     <row r="63">
@@ -1371,8 +1402,8 @@
           <t>NOW LIMPIADOR LAVANDA 1000 L</t>
         </is>
       </c>
-      <c r="C63" s="26" t="n">
-        <v>11490.6</v>
+      <c r="C63" s="31" t="n">
+        <v>11998</v>
       </c>
     </row>
     <row r="64">
@@ -1386,8 +1417,8 @@
           <t>NOW LIMPIADOR MIXTO DE FRUTAS 5 L</t>
         </is>
       </c>
-      <c r="C64" s="26" t="n">
-        <v>116.16</v>
+      <c r="C64" s="31" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="65">
@@ -1401,8 +1432,8 @@
           <t>NOW LIMPIADOR MIXTO DE FRUTAS 10 L</t>
         </is>
       </c>
-      <c r="C65" s="26" t="n">
-        <v>194.04</v>
+      <c r="C65" s="31" t="n">
+        <v>203</v>
       </c>
     </row>
     <row r="66">
@@ -1416,8 +1447,8 @@
           <t>NOW LIMPIADOR DE GRANITO Y MARMOL 1 L</t>
         </is>
       </c>
-      <c r="C66" s="26" t="n">
-        <v>85.8</v>
+      <c r="C66" s="31" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="67">
@@ -1431,8 +1462,8 @@
           <t>NOW LIMPIADOR CONCRETO Y MAMPOSTERIA 1 L</t>
         </is>
       </c>
-      <c r="C67" s="26" t="n">
-        <v>112.2</v>
+      <c r="C67" s="31" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="68">
@@ -1446,8 +1477,8 @@
           <t>NOW LIMPIADOR DE ALFOMBRAS 1 L</t>
         </is>
       </c>
-      <c r="C68" s="26" t="n">
-        <v>87.12</v>
+      <c r="C68" s="31" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="69">
@@ -1461,8 +1492,8 @@
           <t>NOW REMOVEDOR CALCIO SARRO Y OXIDO 1 L</t>
         </is>
       </c>
-      <c r="C69" s="26" t="n">
-        <v>87.12</v>
+      <c r="C69" s="31" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="70">
@@ -1476,8 +1507,8 @@
           <t>NOW JABON LIQUIDO PARA MANOS 5 L</t>
         </is>
       </c>
-      <c r="C70" s="26" t="n">
-        <v>134.64</v>
+      <c r="C70" s="31" t="n">
+        <v>141</v>
       </c>
     </row>
     <row r="71">
@@ -1491,8 +1522,8 @@
           <t>NOW JABON LIQUIDO PARA MANOS 10 L</t>
         </is>
       </c>
-      <c r="C71" s="26" t="n">
-        <v>345.84</v>
+      <c r="C71" s="31" t="n">
+        <v>365</v>
       </c>
     </row>
     <row r="72">
@@ -1506,8 +1537,8 @@
           <t>NOW BLANQUEADOR 20 L</t>
         </is>
       </c>
-      <c r="C72" s="26" t="n">
-        <v>359.04</v>
+      <c r="C72" s="31" t="n">
+        <v>375</v>
       </c>
     </row>
     <row r="73">
@@ -1521,8 +1552,8 @@
           <t>NOW BLANQUEADOR 208 L</t>
         </is>
       </c>
-      <c r="C73" s="26" t="n">
-        <v>3632.64</v>
+      <c r="C73" s="31" t="n">
+        <v>3793</v>
       </c>
     </row>
     <row r="74">
@@ -1536,8 +1567,8 @@
           <t>NOW BLANQUEADOR 1000 L</t>
         </is>
       </c>
-      <c r="C74" s="26" t="n">
-        <v>7505.52</v>
+      <c r="C74" s="31" t="n">
+        <v>7835</v>
       </c>
     </row>
     <row r="75">
@@ -1551,8 +1582,8 @@
           <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 1 L</t>
         </is>
       </c>
-      <c r="C75" s="26" t="n">
-        <v>44.88</v>
+      <c r="C75" s="31" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="76">
@@ -1566,8 +1597,8 @@
           <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 5 L</t>
         </is>
       </c>
-      <c r="C76" s="26" t="n">
-        <v>167.64</v>
+      <c r="C76" s="31" t="n">
+        <v>175</v>
       </c>
     </row>
     <row r="77">
@@ -1581,8 +1612,8 @@
           <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 10 L</t>
         </is>
       </c>
-      <c r="C77" s="26" t="n">
-        <v>282.48</v>
+      <c r="C77" s="31" t="n">
+        <v>295</v>
       </c>
     </row>
     <row r="78">
@@ -1596,8 +1627,8 @@
           <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 208 L</t>
         </is>
       </c>
-      <c r="C78" s="26" t="n">
-        <v>6849.48</v>
+      <c r="C78" s="31" t="n">
+        <v>7148</v>
       </c>
     </row>
     <row r="79">
@@ -1611,8 +1642,8 @@
           <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 1000 L</t>
         </is>
       </c>
-      <c r="C79" s="26" t="n">
-        <v>23432.64</v>
+      <c r="C79" s="31" t="n">
+        <v>24430</v>
       </c>
     </row>
     <row r="80">
@@ -1626,8 +1657,8 @@
           <t>SENSACIONAL SUAVIZANTE VELVET TOUCH 10 L</t>
         </is>
       </c>
-      <c r="C80" s="26" t="n">
-        <v>258.72</v>
+      <c r="C80" s="31" t="n">
+        <v>270</v>
       </c>
     </row>
     <row r="81">
@@ -1641,8 +1672,8 @@
           <t>SENSACIONAL SUAVIZANTE 1 L</t>
         </is>
       </c>
-      <c r="C81" s="26" t="n">
-        <v>39.6</v>
+      <c r="C81" s="31" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="82">
@@ -1656,8 +1687,8 @@
           <t>SENSACIONAL SUAVIZANTE 5 L</t>
         </is>
       </c>
-      <c r="C82" s="26" t="n">
-        <v>132</v>
+      <c r="C82" s="31" t="n">
+        <v>137</v>
       </c>
     </row>
     <row r="83">
@@ -1671,8 +1702,8 @@
           <t>SENSACIONAL SUAVIZANTE 10 L</t>
         </is>
       </c>
-      <c r="C83" s="26" t="n">
-        <v>258.72</v>
+      <c r="C83" s="31" t="n">
+        <v>270</v>
       </c>
     </row>
     <row r="84">
@@ -1686,8 +1717,8 @@
           <t>SENSACIONAL SUAVIZANTE 20 L</t>
         </is>
       </c>
-      <c r="C84" s="26" t="n">
-        <v>591.36</v>
+      <c r="C84" s="31" t="n">
+        <v>617</v>
       </c>
     </row>
     <row r="85">
@@ -1701,8 +1732,8 @@
           <t>SENSACIONAL SUAVIZANTE 208 L</t>
         </is>
       </c>
-      <c r="C85" s="26" t="n">
-        <v>6536.64</v>
+      <c r="C85" s="31" t="n">
+        <v>6816</v>
       </c>
     </row>
     <row r="86">
@@ -1716,11 +1747,3320 @@
           <t>SENSACIONAL SUAVIZANTE 1000 L</t>
         </is>
       </c>
-      <c r="C86" s="27" t="n">
-        <v>19282.56</v>
+      <c r="C86" s="32" t="n">
+        <v>20118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>No. Artículo</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Escala 1 (PDF)</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Escala 2 (PDF - columna 4)</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Escala 3 (PDF)</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Escala 4 (PDF)</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Precio actual Excel</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Precio esperado (Escala 2 + 40%, redondeado hacia abajo)</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Diferencia (Excel original - esperado redondeado)</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>101001-000101</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE MULTIUSOS 1 L</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="D2" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="E2" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F2" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="G2" s="29" t="n">
+        <v>75.23999999999999</v>
+      </c>
+      <c r="H2" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="I2" s="29" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="J2" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>101001-000601</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE MULTIUSOS 5/1 L</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="n">
+        <v>148</v>
+      </c>
+      <c r="D3" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="E3" s="29" t="n">
+        <v>145</v>
+      </c>
+      <c r="F3" s="29" t="n">
+        <v>139</v>
+      </c>
+      <c r="G3" s="29" t="n">
+        <v>195.36</v>
+      </c>
+      <c r="H3" s="33" t="n">
+        <v>205</v>
+      </c>
+      <c r="I3" s="29" t="n">
+        <v>-9.640000000000001</v>
+      </c>
+      <c r="J3" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>101001-002001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE MULTIUSOS 20 L</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="n">
+        <v>440</v>
+      </c>
+      <c r="D4" s="29" t="n">
+        <v>415</v>
+      </c>
+      <c r="E4" s="29" t="n">
+        <v>410</v>
+      </c>
+      <c r="F4" s="29" t="n">
+        <v>394</v>
+      </c>
+      <c r="G4" s="29" t="n">
+        <v>580.8</v>
+      </c>
+      <c r="H4" s="33" t="n">
+        <v>581</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>101001-020801</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE MULTIUSOS 208 L</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>4215</v>
+      </c>
+      <c r="D5" s="29" t="n">
+        <v>4151</v>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>4090</v>
+      </c>
+      <c r="F5" s="29" t="n">
+        <v>3915</v>
+      </c>
+      <c r="G5" s="29" t="n">
+        <v>5563.8</v>
+      </c>
+      <c r="H5" s="33" t="n">
+        <v>5811</v>
+      </c>
+      <c r="I5" s="29" t="n">
+        <v>-247.2</v>
+      </c>
+      <c r="J5" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>101001-100000</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE MULTIUSOS 1000 L</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>11786</v>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>11626</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>11470</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>10873</v>
+      </c>
+      <c r="G6" s="29" t="n">
+        <v>15557.52</v>
+      </c>
+      <c r="H6" s="33" t="n">
+        <v>16276</v>
+      </c>
+      <c r="I6" s="29" t="n">
+        <v>-718.48</v>
+      </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>101003-000101</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE COCINAS 1 L</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="G7" s="29" t="n">
+        <v>75.23999999999999</v>
+      </c>
+      <c r="H7" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="I7" s="29" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="J7" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>101003-020801</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE DE COCINA 208 L</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>4215</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>4151</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>4090</v>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>3915</v>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>5563.8</v>
+      </c>
+      <c r="H8" s="33" t="n">
+        <v>5811</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>-247.2</v>
+      </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>101003-100000</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE DE COCINA 1000 L</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>11786</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>11626</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>11470</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>10873</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>15557.52</v>
+      </c>
+      <c r="H9" s="33" t="n">
+        <v>16276</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>-718.48</v>
+      </c>
+      <c r="J9" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>101004-000101</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NOW VIDRIOS Y SUPERFICIES 1 L</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F10" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="G10" s="29" t="n">
+        <v>75.23999999999999</v>
+      </c>
+      <c r="H10" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>101004-000601</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NOW VIDRIOS Y SUPERFICIES 5/1 L</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>148</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>145</v>
+      </c>
+      <c r="F11" s="29" t="n">
+        <v>139</v>
+      </c>
+      <c r="G11" s="29" t="n">
+        <v>195.36</v>
+      </c>
+      <c r="H11" s="33" t="n">
+        <v>205</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>-9.640000000000001</v>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>101004-020801</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NOW VIDRIOS Y SUPERFICIES 208 L</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>3015</v>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>2963</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>2914</v>
+      </c>
+      <c r="F12" s="29" t="n">
+        <v>2819</v>
+      </c>
+      <c r="G12" s="29" t="n">
+        <v>3979.8</v>
+      </c>
+      <c r="H12" s="33" t="n">
+        <v>4148</v>
+      </c>
+      <c r="I12" s="29" t="n">
+        <v>-168.2</v>
+      </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>101004-100000</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NOW VIDRIOS Y SUPERFICIES 1000 L</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>8216</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>8008</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>7800</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>7488</v>
+      </c>
+      <c r="G13" s="29" t="n">
+        <v>10845.12</v>
+      </c>
+      <c r="H13" s="33" t="n">
+        <v>11211</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>-365.88</v>
+      </c>
+      <c r="J13" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>101006-000101</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE 1 L</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>31</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" s="29" t="n">
+        <v>29</v>
+      </c>
+      <c r="G14" s="29" t="n">
+        <v>42.24</v>
+      </c>
+      <c r="H14" s="33" t="n">
+        <v>43</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>101006-000503</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 5 L MX</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>112</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>105</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>102</v>
+      </c>
+      <c r="F15" s="29" t="n">
+        <v>93</v>
+      </c>
+      <c r="G15" s="29" t="n">
+        <v>147.84</v>
+      </c>
+      <c r="H15" s="33" t="n">
+        <v>147</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J15" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>101006-001000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 10 L</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>211</v>
+      </c>
+      <c r="D16" s="29" t="n">
+        <v>185</v>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>181</v>
+      </c>
+      <c r="F16" s="29" t="n">
+        <v>165</v>
+      </c>
+      <c r="G16" s="29" t="n">
+        <v>278.52</v>
+      </c>
+      <c r="H16" s="33" t="n">
+        <v>259</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>19.52</v>
+      </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>101006-001001</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 10 L DB</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>282</v>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>271</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>267</v>
+      </c>
+      <c r="F17" s="29" t="n">
+        <v>260</v>
+      </c>
+      <c r="G17" s="29" t="n">
+        <v>372.24</v>
+      </c>
+      <c r="H17" s="33" t="n">
+        <v>379</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>-6.76</v>
+      </c>
+      <c r="J17" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>101006-002000</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 20 L</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>480</v>
+      </c>
+      <c r="D18" s="29" t="n">
+        <v>461</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>448</v>
+      </c>
+      <c r="F18" s="29" t="n">
+        <v>420</v>
+      </c>
+      <c r="G18" s="29" t="n">
+        <v>633.6</v>
+      </c>
+      <c r="H18" s="33" t="n">
+        <v>645</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>-11.4</v>
+      </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>101006-020801</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 208 L</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>5274</v>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>5160</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>5045</v>
+      </c>
+      <c r="F19" s="29" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G19" s="29" t="n">
+        <v>6961.68</v>
+      </c>
+      <c r="H19" s="33" t="n">
+        <v>7223</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>-261.32</v>
+      </c>
+      <c r="J19" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>101006-100000</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NOW DETERGENTE LIQ ROPA COLOR 1000 L</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>14075</v>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>13315</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>13035</v>
+      </c>
+      <c r="F20" s="29" t="n">
+        <v>11467</v>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>18579</v>
+      </c>
+      <c r="H20" s="33" t="n">
+        <v>18641</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>-62</v>
+      </c>
+      <c r="J20" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>101008-000101</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>NOW BAÑOS Y AZULEJOS 1 L</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="D21" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F21" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="G21" s="29" t="n">
+        <v>75.23999999999999</v>
+      </c>
+      <c r="H21" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="J21" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>101008-000601</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>NOW BAÑOS Y AZULEJOS 5+1 L</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>148</v>
+      </c>
+      <c r="D22" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>145</v>
+      </c>
+      <c r="F22" s="29" t="n">
+        <v>139</v>
+      </c>
+      <c r="G22" s="29" t="n">
+        <v>195.36</v>
+      </c>
+      <c r="H22" s="33" t="n">
+        <v>205</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>-9.640000000000001</v>
+      </c>
+      <c r="J22" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>101008-002001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>NOW BAÑOS Y AZULEJOS 20 L</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>440</v>
+      </c>
+      <c r="D23" s="29" t="n">
+        <v>415</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>410</v>
+      </c>
+      <c r="F23" s="29" t="n">
+        <v>394</v>
+      </c>
+      <c r="G23" s="29" t="n">
+        <v>580.8</v>
+      </c>
+      <c r="H23" s="33" t="n">
+        <v>581</v>
+      </c>
+      <c r="I23" s="29" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J23" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>101008-020801</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>NOW BAÑOS Y AZULEJOS 208 L</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="n">
+        <v>4215</v>
+      </c>
+      <c r="D24" s="29" t="n">
+        <v>4151</v>
+      </c>
+      <c r="E24" s="29" t="n">
+        <v>4090</v>
+      </c>
+      <c r="F24" s="29" t="n">
+        <v>3915</v>
+      </c>
+      <c r="G24" s="29" t="n">
+        <v>5563.8</v>
+      </c>
+      <c r="H24" s="33" t="n">
+        <v>5811</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>-247.2</v>
+      </c>
+      <c r="J24" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>101008-100000</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NOW BAÑOS Y AZULEJOS 1000 L</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="n">
+        <v>11786</v>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>11626</v>
+      </c>
+      <c r="E25" s="29" t="n">
+        <v>11470</v>
+      </c>
+      <c r="F25" s="29" t="n">
+        <v>10873</v>
+      </c>
+      <c r="G25" s="29" t="n">
+        <v>15557.52</v>
+      </c>
+      <c r="H25" s="33" t="n">
+        <v>16276</v>
+      </c>
+      <c r="I25" s="29" t="n">
+        <v>-718.48</v>
+      </c>
+      <c r="J25" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>101009-001001</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NOW SHAMPOO AUTOMOTRIZ 10 L (PEAD)</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="n">
+        <v>161</v>
+      </c>
+      <c r="D26" s="29" t="n">
+        <v>158</v>
+      </c>
+      <c r="E26" s="29" t="n">
+        <v>155</v>
+      </c>
+      <c r="F26" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="G26" s="29" t="n">
+        <v>212.52</v>
+      </c>
+      <c r="H26" s="33" t="n">
+        <v>221</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>-8.48</v>
+      </c>
+      <c r="J26" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>101009-001002</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NOW SHAMPOO AUTOMOTRIZ 10 L (PET)</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="n">
+        <v>124</v>
+      </c>
+      <c r="D27" s="29" t="n">
+        <v>122</v>
+      </c>
+      <c r="E27" s="29" t="n">
+        <v>120</v>
+      </c>
+      <c r="F27" s="29" t="n">
+        <v>116</v>
+      </c>
+      <c r="G27" s="29" t="n">
+        <v>163.68</v>
+      </c>
+      <c r="H27" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="I27" s="29" t="n">
+        <v>-6.32</v>
+      </c>
+      <c r="J27" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>101009-020800</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NOW SHAMPOO AUTOMOTRIZ 208 L</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="n">
+        <v>3608</v>
+      </c>
+      <c r="D28" s="29" t="n">
+        <v>3546</v>
+      </c>
+      <c r="E28" s="29" t="n">
+        <v>3483</v>
+      </c>
+      <c r="F28" s="29" t="n">
+        <v>3390</v>
+      </c>
+      <c r="G28" s="29" t="n">
+        <v>4762.56</v>
+      </c>
+      <c r="H28" s="33" t="n">
+        <v>4964</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>-201.44</v>
+      </c>
+      <c r="J28" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>101009-100000</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NOW SHAMPOO P/AUTO 1000 L</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="n">
+        <v>8242</v>
+      </c>
+      <c r="D29" s="29" t="n">
+        <v>8101</v>
+      </c>
+      <c r="E29" s="29" t="n">
+        <v>7965</v>
+      </c>
+      <c r="F29" s="29" t="n">
+        <v>7707</v>
+      </c>
+      <c r="G29" s="29" t="n">
+        <v>10879.44</v>
+      </c>
+      <c r="H29" s="33" t="n">
+        <v>11341</v>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>-461.56</v>
+      </c>
+      <c r="J29" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>101010-000101</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>NOW ABRILLANTADOR P/AUTO 1 L ATOM</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="n">
+        <v>47</v>
+      </c>
+      <c r="D30" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="E30" s="29" t="n">
+        <v>45</v>
+      </c>
+      <c r="F30" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="G30" s="29" t="n">
+        <v>62.04</v>
+      </c>
+      <c r="H30" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>-1.96</v>
+      </c>
+      <c r="J30" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>101010-000600</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NOW ABRILLANTADOR P/AUTO 5/1 L</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>207</v>
+      </c>
+      <c r="D31" s="29" t="n">
+        <v>203</v>
+      </c>
+      <c r="E31" s="29" t="n">
+        <v>200</v>
+      </c>
+      <c r="F31" s="29" t="n">
+        <v>194</v>
+      </c>
+      <c r="G31" s="29" t="n">
+        <v>273.24</v>
+      </c>
+      <c r="H31" s="33" t="n">
+        <v>284</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="J31" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>101010-002001</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>NOW ABRILLANTADOR P/AUTO 20 L</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>589</v>
+      </c>
+      <c r="D32" s="29" t="n">
+        <v>580</v>
+      </c>
+      <c r="E32" s="29" t="n">
+        <v>571</v>
+      </c>
+      <c r="F32" s="29" t="n">
+        <v>554</v>
+      </c>
+      <c r="G32" s="29" t="n">
+        <v>777.48</v>
+      </c>
+      <c r="H32" s="33" t="n">
+        <v>812</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>-34.52</v>
+      </c>
+      <c r="J32" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>101010-020801</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NOW ABRILLANTADOR P/AUTO 208 L</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>6156</v>
+      </c>
+      <c r="D33" s="29" t="n">
+        <v>6051</v>
+      </c>
+      <c r="E33" s="29" t="n">
+        <v>5950</v>
+      </c>
+      <c r="F33" s="29" t="n">
+        <v>5757</v>
+      </c>
+      <c r="G33" s="29" t="n">
+        <v>8125.92</v>
+      </c>
+      <c r="H33" s="33" t="n">
+        <v>8471</v>
+      </c>
+      <c r="I33" s="29" t="n">
+        <v>-345.08</v>
+      </c>
+      <c r="J33" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>101010-100000</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NOW ABRILLANTADOR P/AUTO 1000 L</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="n">
+        <v>20876</v>
+      </c>
+      <c r="D34" s="29" t="n">
+        <v>20519</v>
+      </c>
+      <c r="E34" s="29" t="n">
+        <v>20175</v>
+      </c>
+      <c r="F34" s="29" t="n">
+        <v>19520</v>
+      </c>
+      <c r="G34" s="29" t="n">
+        <v>27556.32</v>
+      </c>
+      <c r="H34" s="33" t="n">
+        <v>28726</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>-1169.68</v>
+      </c>
+      <c r="J34" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>101016-000291</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>NOW LAVATRASTES LIMON 2.90 L MX</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="n">
+        <v>104</v>
+      </c>
+      <c r="D35" s="29" t="n">
+        <v>103</v>
+      </c>
+      <c r="E35" s="29" t="n">
+        <v>102</v>
+      </c>
+      <c r="F35" s="29" t="n">
+        <v>95</v>
+      </c>
+      <c r="G35" s="29" t="n">
+        <v>137.28</v>
+      </c>
+      <c r="H35" s="33" t="n">
+        <v>144</v>
+      </c>
+      <c r="I35" s="29" t="n">
+        <v>-6.72</v>
+      </c>
+      <c r="J35" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>101016-000501</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NOW LAVATRASTES LIMON 5 L</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="n">
+        <v>126</v>
+      </c>
+      <c r="D36" s="29" t="n">
+        <v>124</v>
+      </c>
+      <c r="E36" s="29" t="n">
+        <v>122</v>
+      </c>
+      <c r="F36" s="29" t="n">
+        <v>120</v>
+      </c>
+      <c r="G36" s="29" t="n">
+        <v>166.32</v>
+      </c>
+      <c r="H36" s="33" t="n">
+        <v>173</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>-6.68</v>
+      </c>
+      <c r="J36" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>101016-020800</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>NOW LAVATRASTES 208 L</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="n">
+        <v>6042</v>
+      </c>
+      <c r="D37" s="29" t="n">
+        <v>5938</v>
+      </c>
+      <c r="E37" s="29" t="n">
+        <v>5840</v>
+      </c>
+      <c r="F37" s="29" t="n">
+        <v>5658</v>
+      </c>
+      <c r="G37" s="29" t="n">
+        <v>7975.44</v>
+      </c>
+      <c r="H37" s="33" t="n">
+        <v>8313</v>
+      </c>
+      <c r="I37" s="29" t="n">
+        <v>-337.56</v>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>101016-100000</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NOW LAVATRASTES 1000 L</t>
+        </is>
+      </c>
+      <c r="C38" s="29" t="n">
+        <v>19350</v>
+      </c>
+      <c r="D38" s="29" t="n">
+        <v>19017</v>
+      </c>
+      <c r="E38" s="29" t="n">
+        <v>18700</v>
+      </c>
+      <c r="F38" s="29" t="n">
+        <v>18100</v>
+      </c>
+      <c r="G38" s="29" t="n">
+        <v>25542</v>
+      </c>
+      <c r="H38" s="33" t="n">
+        <v>26623</v>
+      </c>
+      <c r="I38" s="29" t="n">
+        <v>-1081</v>
+      </c>
+      <c r="J38" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>101018-000101</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 1 L</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="n">
+        <v>26</v>
+      </c>
+      <c r="D39" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="E39" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="F39" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="G39" s="29" t="n">
+        <v>34.32</v>
+      </c>
+      <c r="H39" s="33" t="n">
+        <v>35</v>
+      </c>
+      <c r="I39" s="29" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="J39" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>101018-000501</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 5 L</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="n">
+        <v>97</v>
+      </c>
+      <c r="D40" s="29" t="n">
+        <v>95</v>
+      </c>
+      <c r="E40" s="29" t="n">
+        <v>94</v>
+      </c>
+      <c r="F40" s="29" t="n">
+        <v>83</v>
+      </c>
+      <c r="G40" s="29" t="n">
+        <v>128.04</v>
+      </c>
+      <c r="H40" s="33" t="n">
+        <v>133</v>
+      </c>
+      <c r="I40" s="29" t="n">
+        <v>-4.96</v>
+      </c>
+      <c r="J40" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>101018-001000</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 10 L</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="n">
+        <v>177</v>
+      </c>
+      <c r="D41" s="29" t="n">
+        <v>174</v>
+      </c>
+      <c r="E41" s="29" t="n">
+        <v>172</v>
+      </c>
+      <c r="F41" s="29" t="n">
+        <v>152</v>
+      </c>
+      <c r="G41" s="29" t="n">
+        <v>233.64</v>
+      </c>
+      <c r="H41" s="33" t="n">
+        <v>243</v>
+      </c>
+      <c r="I41" s="29" t="n">
+        <v>-9.359999999999999</v>
+      </c>
+      <c r="J41" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>101018-002000</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 20 L</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="n">
+        <v>359</v>
+      </c>
+      <c r="D42" s="29" t="n">
+        <v>353</v>
+      </c>
+      <c r="E42" s="29" t="n">
+        <v>347</v>
+      </c>
+      <c r="F42" s="29" t="n">
+        <v>335</v>
+      </c>
+      <c r="G42" s="29" t="n">
+        <v>473.88</v>
+      </c>
+      <c r="H42" s="33" t="n">
+        <v>494</v>
+      </c>
+      <c r="I42" s="29" t="n">
+        <v>-20.12</v>
+      </c>
+      <c r="J42" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>101018-020800</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 208 L</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="n">
+        <v>4373</v>
+      </c>
+      <c r="D43" s="29" t="n">
+        <v>4301</v>
+      </c>
+      <c r="E43" s="29" t="n">
+        <v>4228</v>
+      </c>
+      <c r="F43" s="29" t="n">
+        <v>4093</v>
+      </c>
+      <c r="G43" s="29" t="n">
+        <v>5772.36</v>
+      </c>
+      <c r="H43" s="33" t="n">
+        <v>6021</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <v>-248.64</v>
+      </c>
+      <c r="J43" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>101018-100000</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR PINO 1000 L</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="n">
+        <v>12376</v>
+      </c>
+      <c r="D44" s="29" t="n">
+        <v>12168</v>
+      </c>
+      <c r="E44" s="29" t="n">
+        <v>11960</v>
+      </c>
+      <c r="F44" s="29" t="n">
+        <v>11252</v>
+      </c>
+      <c r="G44" s="29" t="n">
+        <v>16336.32</v>
+      </c>
+      <c r="H44" s="33" t="n">
+        <v>17035</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>-698.6799999999999</v>
+      </c>
+      <c r="J44" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>101019-000101</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR MANZANA CANELA 1 L</t>
+        </is>
+      </c>
+      <c r="C45" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="D45" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="E45" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="F45" s="29" t="n">
+        <v>21</v>
+      </c>
+      <c r="G45" s="29" t="n">
+        <v>31.68</v>
+      </c>
+      <c r="H45" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="I45" s="29" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="J45" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>101019-000501</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR MANZANA CANELA 5 L</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="n">
+        <v>75</v>
+      </c>
+      <c r="D46" s="29" t="n">
+        <v>74</v>
+      </c>
+      <c r="E46" s="29" t="n">
+        <v>73</v>
+      </c>
+      <c r="F46" s="29" t="n">
+        <v>70</v>
+      </c>
+      <c r="G46" s="29" t="n">
+        <v>99</v>
+      </c>
+      <c r="H46" s="33" t="n">
+        <v>103</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>-4</v>
+      </c>
+      <c r="J46" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>101019-001001</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR MANZANA CANELA 10 L</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="n">
+        <v>122</v>
+      </c>
+      <c r="D47" s="29" t="n">
+        <v>120</v>
+      </c>
+      <c r="E47" s="29" t="n">
+        <v>118</v>
+      </c>
+      <c r="F47" s="29" t="n">
+        <v>114</v>
+      </c>
+      <c r="G47" s="29" t="n">
+        <v>161.04</v>
+      </c>
+      <c r="H47" s="33" t="n">
+        <v>168</v>
+      </c>
+      <c r="I47" s="29" t="n">
+        <v>-6.96</v>
+      </c>
+      <c r="J47" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>101021-001001</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>NOW QUITAMANCHAS GEL 10 L</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="n">
+        <v>222</v>
+      </c>
+      <c r="D48" s="29" t="n">
+        <v>219</v>
+      </c>
+      <c r="E48" s="29" t="n">
+        <v>215</v>
+      </c>
+      <c r="F48" s="29" t="n">
+        <v>205</v>
+      </c>
+      <c r="G48" s="29" t="n">
+        <v>293.04</v>
+      </c>
+      <c r="H48" s="33" t="n">
+        <v>306</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>-12.96</v>
+      </c>
+      <c r="J48" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>101021-020800</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>NOW QUITAMANCHAS 208 L</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="n">
+        <v>4160</v>
+      </c>
+      <c r="D49" s="29" t="n">
+        <v>4108</v>
+      </c>
+      <c r="E49" s="29" t="n">
+        <v>4056</v>
+      </c>
+      <c r="F49" s="29" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G49" s="29" t="n">
+        <v>5491.2</v>
+      </c>
+      <c r="H49" s="33" t="n">
+        <v>5751</v>
+      </c>
+      <c r="I49" s="29" t="n">
+        <v>-259.8</v>
+      </c>
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>101021-100000</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>NOW QUITAMANCHAS GEL 1000 L</t>
+        </is>
+      </c>
+      <c r="C50" s="29" t="n">
+        <v>11399</v>
+      </c>
+      <c r="D50" s="29" t="n">
+        <v>11212</v>
+      </c>
+      <c r="E50" s="29" t="n">
+        <v>11025</v>
+      </c>
+      <c r="F50" s="29" t="n">
+        <v>10678</v>
+      </c>
+      <c r="G50" s="29" t="n">
+        <v>15046.68</v>
+      </c>
+      <c r="H50" s="33" t="n">
+        <v>15696</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>-649.3200000000001</v>
+      </c>
+      <c r="J50" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>101022-000501</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE AUTOMOTRIZ 5 L</t>
+        </is>
+      </c>
+      <c r="C51" s="29" t="n">
+        <v>166</v>
+      </c>
+      <c r="D51" s="29" t="n">
+        <v>160</v>
+      </c>
+      <c r="E51" s="29" t="n">
+        <v>159</v>
+      </c>
+      <c r="F51" s="29" t="n">
+        <v>140</v>
+      </c>
+      <c r="G51" s="29" t="n">
+        <v>219.12</v>
+      </c>
+      <c r="H51" s="33" t="n">
+        <v>224</v>
+      </c>
+      <c r="I51" s="29" t="n">
+        <v>-4.88</v>
+      </c>
+      <c r="J51" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>101022-002001</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE AUTOMOTRIZ 20 L</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="n">
+        <v>645</v>
+      </c>
+      <c r="D52" s="29" t="n">
+        <v>635</v>
+      </c>
+      <c r="E52" s="29" t="n">
+        <v>624</v>
+      </c>
+      <c r="F52" s="29" t="n">
+        <v>552</v>
+      </c>
+      <c r="G52" s="29" t="n">
+        <v>851.4</v>
+      </c>
+      <c r="H52" s="33" t="n">
+        <v>889</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>-37.6</v>
+      </c>
+      <c r="J52" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>101022-020800</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE AUTOMOTRIZ 208 L</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="n">
+        <v>6448</v>
+      </c>
+      <c r="D53" s="29" t="n">
+        <v>6344</v>
+      </c>
+      <c r="E53" s="29" t="n">
+        <v>6240</v>
+      </c>
+      <c r="F53" s="29" t="n">
+        <v>5460</v>
+      </c>
+      <c r="G53" s="29" t="n">
+        <v>8511.360000000001</v>
+      </c>
+      <c r="H53" s="33" t="n">
+        <v>8881</v>
+      </c>
+      <c r="I53" s="29" t="n">
+        <v>-369.64</v>
+      </c>
+      <c r="J53" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>101022-100000</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>NOW DESENGRASANTE AUTOMOTRIZ 1000 L</t>
+        </is>
+      </c>
+      <c r="C54" s="29" t="n">
+        <v>24753</v>
+      </c>
+      <c r="D54" s="29" t="n">
+        <v>24450</v>
+      </c>
+      <c r="E54" s="29" t="n">
+        <v>23920</v>
+      </c>
+      <c r="F54" s="29" t="n">
+        <v>21008</v>
+      </c>
+      <c r="G54" s="29" t="n">
+        <v>32673.96</v>
+      </c>
+      <c r="H54" s="33" t="n">
+        <v>34230</v>
+      </c>
+      <c r="I54" s="29" t="n">
+        <v>-1556.04</v>
+      </c>
+      <c r="J54" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>101025-000101</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR BRISA MARINA 1 L</t>
+        </is>
+      </c>
+      <c r="C55" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="D55" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="E55" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="F55" s="29" t="n">
+        <v>21</v>
+      </c>
+      <c r="G55" s="29" t="n">
+        <v>31.68</v>
+      </c>
+      <c r="H55" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="I55" s="29" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="J55" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>101025-000502</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR BRISA MARINA 5 L</t>
+        </is>
+      </c>
+      <c r="C56" s="29" t="n">
+        <v>75</v>
+      </c>
+      <c r="D56" s="29" t="n">
+        <v>74</v>
+      </c>
+      <c r="E56" s="29" t="n">
+        <v>73</v>
+      </c>
+      <c r="F56" s="29" t="n">
+        <v>70</v>
+      </c>
+      <c r="G56" s="29" t="n">
+        <v>99</v>
+      </c>
+      <c r="H56" s="33" t="n">
+        <v>103</v>
+      </c>
+      <c r="I56" s="29" t="n">
+        <v>-4</v>
+      </c>
+      <c r="J56" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>101025-001001</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR BRISA DE MAR 10 L</t>
+        </is>
+      </c>
+      <c r="C57" s="29" t="n">
+        <v>122</v>
+      </c>
+      <c r="D57" s="29" t="n">
+        <v>120</v>
+      </c>
+      <c r="E57" s="29" t="n">
+        <v>118</v>
+      </c>
+      <c r="F57" s="29" t="n">
+        <v>114</v>
+      </c>
+      <c r="G57" s="29" t="n">
+        <v>161.04</v>
+      </c>
+      <c r="H57" s="33" t="n">
+        <v>168</v>
+      </c>
+      <c r="I57" s="29" t="n">
+        <v>-6.96</v>
+      </c>
+      <c r="J57" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>101027-000101</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 1 L</t>
+        </is>
+      </c>
+      <c r="C58" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="D58" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="E58" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="F58" s="29" t="n">
+        <v>21</v>
+      </c>
+      <c r="G58" s="29" t="n">
+        <v>31.68</v>
+      </c>
+      <c r="H58" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="J58" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>101027-000502</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 5 L</t>
+        </is>
+      </c>
+      <c r="C59" s="29" t="n">
+        <v>71</v>
+      </c>
+      <c r="D59" s="29" t="n">
+        <v>70</v>
+      </c>
+      <c r="E59" s="29" t="n">
+        <v>69</v>
+      </c>
+      <c r="F59" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="G59" s="29" t="n">
+        <v>93.72</v>
+      </c>
+      <c r="H59" s="33" t="n">
+        <v>98</v>
+      </c>
+      <c r="I59" s="29" t="n">
+        <v>-4.28</v>
+      </c>
+      <c r="J59" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>101027-001000</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 10 L</t>
+        </is>
+      </c>
+      <c r="C60" s="29" t="n">
+        <v>117</v>
+      </c>
+      <c r="D60" s="29" t="n">
+        <v>115</v>
+      </c>
+      <c r="E60" s="29" t="n">
+        <v>113</v>
+      </c>
+      <c r="F60" s="29" t="n">
+        <v>111</v>
+      </c>
+      <c r="G60" s="29" t="n">
+        <v>154.44</v>
+      </c>
+      <c r="H60" s="33" t="n">
+        <v>161</v>
+      </c>
+      <c r="I60" s="29" t="n">
+        <v>-6.56</v>
+      </c>
+      <c r="J60" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>101027-002000</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 20 L</t>
+        </is>
+      </c>
+      <c r="C61" s="29" t="n">
+        <v>281</v>
+      </c>
+      <c r="D61" s="29" t="n">
+        <v>276</v>
+      </c>
+      <c r="E61" s="29" t="n">
+        <v>273</v>
+      </c>
+      <c r="F61" s="29" t="n">
+        <v>262</v>
+      </c>
+      <c r="G61" s="29" t="n">
+        <v>370.92</v>
+      </c>
+      <c r="H61" s="33" t="n">
+        <v>386</v>
+      </c>
+      <c r="I61" s="29" t="n">
+        <v>-15.08</v>
+      </c>
+      <c r="J61" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>101027-020800</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 208 L</t>
+        </is>
+      </c>
+      <c r="C62" s="29" t="n">
+        <v>3542</v>
+      </c>
+      <c r="D62" s="29" t="n">
+        <v>3483</v>
+      </c>
+      <c r="E62" s="29" t="n">
+        <v>3421</v>
+      </c>
+      <c r="F62" s="29" t="n">
+        <v>3313</v>
+      </c>
+      <c r="G62" s="29" t="n">
+        <v>4675.44</v>
+      </c>
+      <c r="H62" s="33" t="n">
+        <v>4876</v>
+      </c>
+      <c r="I62" s="29" t="n">
+        <v>-200.56</v>
+      </c>
+      <c r="J62" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>101027-100000</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR LAVANDA 1000 L</t>
+        </is>
+      </c>
+      <c r="C63" s="29" t="n">
+        <v>8705</v>
+      </c>
+      <c r="D63" s="29" t="n">
+        <v>8570</v>
+      </c>
+      <c r="E63" s="29" t="n">
+        <v>8445</v>
+      </c>
+      <c r="F63" s="29" t="n">
+        <v>8320</v>
+      </c>
+      <c r="G63" s="29" t="n">
+        <v>11490.6</v>
+      </c>
+      <c r="H63" s="33" t="n">
+        <v>11998</v>
+      </c>
+      <c r="I63" s="29" t="n">
+        <v>-507.4</v>
+      </c>
+      <c r="J63" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>101028-000501</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR MIXTO DE FRUTAS 5 L</t>
+        </is>
+      </c>
+      <c r="C64" s="29" t="n">
+        <v>88</v>
+      </c>
+      <c r="D64" s="29" t="n">
+        <v>86</v>
+      </c>
+      <c r="E64" s="29" t="n">
+        <v>85</v>
+      </c>
+      <c r="F64" s="29" t="n">
+        <v>76</v>
+      </c>
+      <c r="G64" s="29" t="n">
+        <v>116.16</v>
+      </c>
+      <c r="H64" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="I64" s="29" t="n">
+        <v>-3.84</v>
+      </c>
+      <c r="J64" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>101028-001001</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR MIXTO DE FRUTAS 10 L</t>
+        </is>
+      </c>
+      <c r="C65" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="D65" s="29" t="n">
+        <v>145</v>
+      </c>
+      <c r="E65" s="29" t="n">
+        <v>143</v>
+      </c>
+      <c r="F65" s="29" t="n">
+        <v>127</v>
+      </c>
+      <c r="G65" s="29" t="n">
+        <v>194.04</v>
+      </c>
+      <c r="H65" s="33" t="n">
+        <v>203</v>
+      </c>
+      <c r="I65" s="29" t="n">
+        <v>-8.960000000000001</v>
+      </c>
+      <c r="J65" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>101029-000101</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR DE GRANITO Y MARMOL 1 L</t>
+        </is>
+      </c>
+      <c r="C66" s="29" t="n">
+        <v>65</v>
+      </c>
+      <c r="D66" s="29" t="n">
+        <v>64</v>
+      </c>
+      <c r="E66" s="29" t="n">
+        <v>63</v>
+      </c>
+      <c r="F66" s="29" t="n">
+        <v>57</v>
+      </c>
+      <c r="G66" s="29" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="H66" s="33" t="n">
+        <v>89</v>
+      </c>
+      <c r="I66" s="29" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="J66" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>101030-000101</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR CONCRETO Y MAMPOSTERIA 1 L</t>
+        </is>
+      </c>
+      <c r="C67" s="29" t="n">
+        <v>85</v>
+      </c>
+      <c r="D67" s="29" t="n">
+        <v>84</v>
+      </c>
+      <c r="E67" s="29" t="n">
+        <v>83</v>
+      </c>
+      <c r="F67" s="29" t="n">
+        <v>74</v>
+      </c>
+      <c r="G67" s="29" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="H67" s="33" t="n">
+        <v>117</v>
+      </c>
+      <c r="I67" s="29" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="J67" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>101031-000101</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>NOW LIMPIADOR DE ALFOMBRAS 1 L</t>
+        </is>
+      </c>
+      <c r="C68" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="D68" s="29" t="n">
+        <v>64</v>
+      </c>
+      <c r="E68" s="29" t="n">
+        <v>63</v>
+      </c>
+      <c r="F68" s="29" t="n">
+        <v>59</v>
+      </c>
+      <c r="G68" s="29" t="n">
+        <v>87.12</v>
+      </c>
+      <c r="H68" s="33" t="n">
+        <v>89</v>
+      </c>
+      <c r="I68" s="29" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="J68" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>101032-000101</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NOW REMOVEDOR CALCIO SARRO Y OXIDO 1 L</t>
+        </is>
+      </c>
+      <c r="C69" s="29" t="n">
+        <v>66</v>
+      </c>
+      <c r="D69" s="29" t="n">
+        <v>64</v>
+      </c>
+      <c r="E69" s="29" t="n">
+        <v>63</v>
+      </c>
+      <c r="F69" s="29" t="n">
+        <v>59</v>
+      </c>
+      <c r="G69" s="29" t="n">
+        <v>87.12</v>
+      </c>
+      <c r="H69" s="33" t="n">
+        <v>89</v>
+      </c>
+      <c r="I69" s="29" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="J69" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>101041-000500</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>NOW JABON LIQUIDO PARA MANOS 5 L</t>
+        </is>
+      </c>
+      <c r="C70" s="29" t="n">
+        <v>102</v>
+      </c>
+      <c r="D70" s="29" t="n">
+        <v>101</v>
+      </c>
+      <c r="E70" s="29" t="n">
+        <v>85</v>
+      </c>
+      <c r="F70" s="29" t="n">
+        <v>82</v>
+      </c>
+      <c r="G70" s="29" t="n">
+        <v>134.64</v>
+      </c>
+      <c r="H70" s="33" t="n">
+        <v>141</v>
+      </c>
+      <c r="I70" s="29" t="n">
+        <v>-6.36</v>
+      </c>
+      <c r="J70" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>101041-001000</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>NOW JABON LIQUIDO PARA MANOS 10 L</t>
+        </is>
+      </c>
+      <c r="C71" s="29" t="n">
+        <v>262</v>
+      </c>
+      <c r="D71" s="29" t="n">
+        <v>261</v>
+      </c>
+      <c r="E71" s="29" t="n">
+        <v>214</v>
+      </c>
+      <c r="F71" s="29" t="n">
+        <v>206</v>
+      </c>
+      <c r="G71" s="29" t="n">
+        <v>345.84</v>
+      </c>
+      <c r="H71" s="33" t="n">
+        <v>365</v>
+      </c>
+      <c r="I71" s="29" t="n">
+        <v>-19.16</v>
+      </c>
+      <c r="J71" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>101042-002000</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>NOW BLANQUEADOR 20 L</t>
+        </is>
+      </c>
+      <c r="C72" s="29" t="n">
+        <v>272</v>
+      </c>
+      <c r="D72" s="29" t="n">
+        <v>268</v>
+      </c>
+      <c r="E72" s="29" t="n">
+        <v>265</v>
+      </c>
+      <c r="F72" s="29" t="n">
+        <v>241</v>
+      </c>
+      <c r="G72" s="29" t="n">
+        <v>359.04</v>
+      </c>
+      <c r="H72" s="33" t="n">
+        <v>375</v>
+      </c>
+      <c r="I72" s="29" t="n">
+        <v>-15.96</v>
+      </c>
+      <c r="J72" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>101042-020800</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>NOW BLANQUEADOR 208 L</t>
+        </is>
+      </c>
+      <c r="C73" s="29" t="n">
+        <v>2752</v>
+      </c>
+      <c r="D73" s="29" t="n">
+        <v>2710</v>
+      </c>
+      <c r="E73" s="29" t="n">
+        <v>2668</v>
+      </c>
+      <c r="F73" s="29" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G73" s="29" t="n">
+        <v>3632.64</v>
+      </c>
+      <c r="H73" s="33" t="n">
+        <v>3793</v>
+      </c>
+      <c r="I73" s="29" t="n">
+        <v>-160.36</v>
+      </c>
+      <c r="J73" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>101042-100000</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>NOW BLANQUEADOR 1000 L</t>
+        </is>
+      </c>
+      <c r="C74" s="29" t="n">
+        <v>5686</v>
+      </c>
+      <c r="D74" s="29" t="n">
+        <v>5597</v>
+      </c>
+      <c r="E74" s="29" t="n">
+        <v>5512</v>
+      </c>
+      <c r="F74" s="29" t="n">
+        <v>4685</v>
+      </c>
+      <c r="G74" s="29" t="n">
+        <v>7505.52</v>
+      </c>
+      <c r="H74" s="33" t="n">
+        <v>7835</v>
+      </c>
+      <c r="I74" s="29" t="n">
+        <v>-329.48</v>
+      </c>
+      <c r="J74" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>102003-000101</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 1 L</t>
+        </is>
+      </c>
+      <c r="C75" s="29" t="n">
+        <v>34</v>
+      </c>
+      <c r="D75" s="29" t="n">
+        <v>33</v>
+      </c>
+      <c r="E75" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="F75" s="29" t="n">
+        <v>31</v>
+      </c>
+      <c r="G75" s="29" t="n">
+        <v>44.88</v>
+      </c>
+      <c r="H75" s="33" t="n">
+        <v>46</v>
+      </c>
+      <c r="I75" s="29" t="n">
+        <v>-1.12</v>
+      </c>
+      <c r="J75" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>102003-000501</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 5 L</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="n">
+        <v>127</v>
+      </c>
+      <c r="D76" s="29" t="n">
+        <v>125</v>
+      </c>
+      <c r="E76" s="29" t="n">
+        <v>123</v>
+      </c>
+      <c r="F76" s="29" t="n">
+        <v>121</v>
+      </c>
+      <c r="G76" s="29" t="n">
+        <v>167.64</v>
+      </c>
+      <c r="H76" s="33" t="n">
+        <v>175</v>
+      </c>
+      <c r="I76" s="29" t="n">
+        <v>-7.36</v>
+      </c>
+      <c r="J76" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>102003-001001</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 10 L</t>
+        </is>
+      </c>
+      <c r="C77" s="29" t="n">
+        <v>214</v>
+      </c>
+      <c r="D77" s="29" t="n">
+        <v>211</v>
+      </c>
+      <c r="E77" s="29" t="n">
+        <v>207</v>
+      </c>
+      <c r="F77" s="29" t="n">
+        <v>201</v>
+      </c>
+      <c r="G77" s="29" t="n">
+        <v>282.48</v>
+      </c>
+      <c r="H77" s="33" t="n">
+        <v>295</v>
+      </c>
+      <c r="I77" s="29" t="n">
+        <v>-12.52</v>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>102003-020801</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 208 L</t>
+        </is>
+      </c>
+      <c r="C78" s="29" t="n">
+        <v>5189</v>
+      </c>
+      <c r="D78" s="29" t="n">
+        <v>5106</v>
+      </c>
+      <c r="E78" s="29" t="n">
+        <v>5018</v>
+      </c>
+      <c r="F78" s="29" t="n">
+        <v>4856</v>
+      </c>
+      <c r="G78" s="29" t="n">
+        <v>6849.48</v>
+      </c>
+      <c r="H78" s="33" t="n">
+        <v>7148</v>
+      </c>
+      <c r="I78" s="29" t="n">
+        <v>-298.52</v>
+      </c>
+      <c r="J78" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>102003-100000</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE TOQUE DE SEDA 1000 L</t>
+        </is>
+      </c>
+      <c r="C79" s="29" t="n">
+        <v>17752</v>
+      </c>
+      <c r="D79" s="29" t="n">
+        <v>17450</v>
+      </c>
+      <c r="E79" s="29" t="n">
+        <v>17159</v>
+      </c>
+      <c r="F79" s="29" t="n">
+        <v>16597</v>
+      </c>
+      <c r="G79" s="29" t="n">
+        <v>23432.64</v>
+      </c>
+      <c r="H79" s="33" t="n">
+        <v>24430</v>
+      </c>
+      <c r="I79" s="29" t="n">
+        <v>-997.36</v>
+      </c>
+      <c r="J79" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>102007-001001</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE VELVET TOUCH 10 L</t>
+        </is>
+      </c>
+      <c r="C80" s="29" t="n">
+        <v>196</v>
+      </c>
+      <c r="D80" s="29" t="n">
+        <v>193</v>
+      </c>
+      <c r="E80" s="29" t="n">
+        <v>190</v>
+      </c>
+      <c r="F80" s="29" t="n">
+        <v>171</v>
+      </c>
+      <c r="G80" s="29" t="n">
+        <v>258.72</v>
+      </c>
+      <c r="H80" s="33" t="n">
+        <v>270</v>
+      </c>
+      <c r="I80" s="29" t="n">
+        <v>-11.28</v>
+      </c>
+      <c r="J80" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>102026-000101</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 1 L</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="D81" s="29" t="n">
+        <v>29</v>
+      </c>
+      <c r="E81" s="29" t="n">
+        <v>27</v>
+      </c>
+      <c r="F81" s="29" t="n">
+        <v>26</v>
+      </c>
+      <c r="G81" s="29" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="H81" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="I81" s="29" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="J81" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>102026-000501</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 5 L</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="n">
+        <v>100</v>
+      </c>
+      <c r="D82" s="29" t="n">
+        <v>98</v>
+      </c>
+      <c r="E82" s="29" t="n">
+        <v>97</v>
+      </c>
+      <c r="F82" s="29" t="n">
+        <v>91</v>
+      </c>
+      <c r="G82" s="29" t="n">
+        <v>132</v>
+      </c>
+      <c r="H82" s="33" t="n">
+        <v>137</v>
+      </c>
+      <c r="I82" s="29" t="n">
+        <v>-5</v>
+      </c>
+      <c r="J82" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>102026-001001</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 10 L</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="n">
+        <v>196</v>
+      </c>
+      <c r="D83" s="29" t="n">
+        <v>193</v>
+      </c>
+      <c r="E83" s="29" t="n">
+        <v>190</v>
+      </c>
+      <c r="F83" s="29" t="n">
+        <v>171</v>
+      </c>
+      <c r="G83" s="29" t="n">
+        <v>258.72</v>
+      </c>
+      <c r="H83" s="33" t="n">
+        <v>270</v>
+      </c>
+      <c r="I83" s="29" t="n">
+        <v>-11.28</v>
+      </c>
+      <c r="J83" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>102026-002001</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 20 L</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="n">
+        <v>448</v>
+      </c>
+      <c r="D84" s="29" t="n">
+        <v>441</v>
+      </c>
+      <c r="E84" s="29" t="n">
+        <v>434</v>
+      </c>
+      <c r="F84" s="29" t="n">
+        <v>422</v>
+      </c>
+      <c r="G84" s="29" t="n">
+        <v>591.36</v>
+      </c>
+      <c r="H84" s="33" t="n">
+        <v>617</v>
+      </c>
+      <c r="I84" s="29" t="n">
+        <v>-25.64</v>
+      </c>
+      <c r="J84" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>102026-020801</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 208 L</t>
+        </is>
+      </c>
+      <c r="C85" s="29" t="n">
+        <v>4952</v>
+      </c>
+      <c r="D85" s="29" t="n">
+        <v>4869</v>
+      </c>
+      <c r="E85" s="29" t="n">
+        <v>4796</v>
+      </c>
+      <c r="F85" s="29" t="n">
+        <v>4646</v>
+      </c>
+      <c r="G85" s="29" t="n">
+        <v>6536.64</v>
+      </c>
+      <c r="H85" s="33" t="n">
+        <v>6816</v>
+      </c>
+      <c r="I85" s="29" t="n">
+        <v>-279.36</v>
+      </c>
+      <c r="J85" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>102026-100000</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SENSACIONAL SUAVIZANTE 1000 L</t>
+        </is>
+      </c>
+      <c r="C86" s="29" t="n">
+        <v>14608</v>
+      </c>
+      <c r="D86" s="29" t="n">
+        <v>14370</v>
+      </c>
+      <c r="E86" s="29" t="n">
+        <v>14140</v>
+      </c>
+      <c r="F86" s="29" t="n">
+        <v>13704</v>
+      </c>
+      <c r="G86" s="29" t="n">
+        <v>19282.56</v>
+      </c>
+      <c r="H86" s="33" t="n">
+        <v>20118</v>
+      </c>
+      <c r="I86" s="29" t="n">
+        <v>-835.4400000000001</v>
+      </c>
+      <c r="J86" s="30" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J86"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>